<commit_message>
Actualización automática 2026-09-14 08:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1185,10 +1185,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>0</v>
+        <v>2361.15</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>0</v>
+        <v>205.37</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>2495.93</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>0</v>
+        <v>1210.28</v>
       </c>
       <c r="I24" s="2" t="n">
         <v>0</v>
@@ -2026,32 +2026,32 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
+          <t>3 de 24</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
           <t>1 de 24</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>0 de 24</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>0 de 24</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>0 de 24</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>2 de 24</t>
+          <t>3 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2431,7 +2431,7 @@
         <v>6827.71</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0</v>
+        <v>5062.45</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>5000</v>
@@ -2674,7 +2674,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0</v>
+        <v>1210.28</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>3000</v>
@@ -2718,7 +2718,7 @@
         <v>43619.47</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>6681.43</v>
+        <v>12954.16</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>
@@ -2913,13 +2913,13 @@
         <v>5190</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2801.71</v>
+        <v>6373.14</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>2388.29</v>
+        <v>-1183.14</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>0.5398285163776493</v>
+        <v>1.227965317919075</v>
       </c>
     </row>
     <row r="8">
@@ -2937,13 +2937,13 @@
         <v>963</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>0</v>
+        <v>205.37</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>963</v>
+        <v>757.63</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>0.2132606438213915</v>
       </c>
     </row>
     <row r="9">
@@ -3081,13 +3081,13 @@
         <v>36556</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>4018.81</v>
+        <v>6514.74</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>32537.19</v>
+        <v>30041.26</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.109935715067294</v>
+        <v>0.1782126053178685</v>
       </c>
     </row>
     <row r="15">
@@ -3124,13 +3124,13 @@
         <v>51596.88</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>6681.43</v>
+        <v>12954.16</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>44915.45</v>
+        <v>38642.72</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.1294929073230784</v>
+        <v>0.251064793065007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-22 12:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1494,7 +1494,7 @@
         <v>0</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>1263.36</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2512,7 +2512,7 @@
         <v>3252.74</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1550.24</v>
+        <v>2813.6</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6000</v>
@@ -2718,7 +2718,7 @@
         <v>43619.47</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>14800.26</v>
+        <v>16063.62</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>
@@ -2742,7 +2742,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3009,13 +3009,13 @@
         <v>407</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>1263.36</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>407</v>
+        <v>-856.3599999999999</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>3.104078624078624</v>
       </c>
     </row>
     <row r="12">
@@ -3124,13 +3124,13 @@
         <v>51596.88</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>14800.26</v>
+        <v>16063.62</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>36796.62</v>
+        <v>35533.26</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2868440882471963</v>
+        <v>0.3113292896779805</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-24 12:30:17
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1185,10 +1185,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>2361.15</v>
+        <v>4187.7</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>595.65</v>
+        <v>735.05</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0</v>
@@ -1905,7 +1905,7 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>1210.28</v>
+        <v>1774.58</v>
       </c>
       <c r="I24" s="2" t="n">
         <v>0</v>
@@ -2431,7 +2431,7 @@
         <v>6827.71</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>6973.37</v>
+        <v>8939.32</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>5000</v>
@@ -2674,7 +2674,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>1210.28</v>
+        <v>1774.58</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>3000</v>
@@ -2718,7 +2718,7 @@
         <v>43619.47</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>16063.62</v>
+        <v>18593.87</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>
@@ -2913,13 +2913,13 @@
         <v>5190</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>6373.14</v>
+        <v>8763.99</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-1183.14</v>
+        <v>-3573.99</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.227965317919075</v>
+        <v>1.688630057803468</v>
       </c>
     </row>
     <row r="8">
@@ -2937,13 +2937,13 @@
         <v>963</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>595.65</v>
+        <v>735.05</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>367.35</v>
+        <v>227.95</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.6185358255451713</v>
+        <v>0.7632917964693665</v>
       </c>
     </row>
     <row r="9">
@@ -3124,13 +3124,13 @@
         <v>51596.88</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>16063.62</v>
+        <v>18593.87</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>35533.26</v>
+        <v>33003.01</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3113292896779805</v>
+        <v>0.3603681075289823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 13:30:17
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1134,7 +1134,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0</v>
+        <v>355.32</v>
       </c>
       <c r="L11" s="2" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0</v>
+        <v>355.32</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>2000</v>
@@ -2718,7 +2718,7 @@
         <v>43619.47</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>17330.51</v>
+        <v>17685.83</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>
@@ -2742,7 +2742,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3009,13 +3009,13 @@
         <v>407</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0</v>
+        <v>355.32</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>407</v>
+        <v>51.68000000000001</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>0</v>
+        <v>0.873022113022113</v>
       </c>
     </row>
     <row r="12">
@@ -3124,13 +3124,13 @@
         <v>51596.88</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>17330.51</v>
+        <v>17685.83</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>34266.37</v>
+        <v>33911.05</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3358829060981981</v>
+        <v>0.3427693690006062</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-28 17:30:18
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1488,7 +1488,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>0</v>
+        <v>1029.61</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0</v>
@@ -1497,7 +1497,7 @@
         <v>0</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>0</v>
+        <v>3245.36</v>
       </c>
       <c r="M17" s="2" t="n">
         <v>1550.24</v>
@@ -1965,10 +1965,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>0</v>
+        <v>4672.8</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>3656.3</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0</v>
@@ -2026,27 +2026,27 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
+          <t>4 de 24</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
           <t>3 de 24</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>0 de 24</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>1 de 24</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>1 de 24</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>0 de 24</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
@@ -2512,7 +2512,7 @@
         <v>3252.74</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>1550.24</v>
+        <v>5825.21</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6000</v>
@@ -2701,7 +2701,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0</v>
+        <v>8329.1</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>6000</v>
@@ -2718,7 +2718,7 @@
         <v>43619.47</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>17685.83</v>
+        <v>30289.9</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>
@@ -2741,7 +2741,7 @@
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
@@ -2913,13 +2913,13 @@
         <v>5190</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>8763.99</v>
+        <v>13436.79</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-3573.99</v>
+        <v>-8246.790000000001</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.688630057803468</v>
+        <v>2.588976878612717</v>
       </c>
     </row>
     <row r="8">
@@ -2937,13 +2937,13 @@
         <v>963</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>735.05</v>
+        <v>5420.96</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>227.95</v>
+        <v>-4457.96</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.7632917964693665</v>
+        <v>5.629241952232606</v>
       </c>
     </row>
     <row r="9">
@@ -3057,13 +3057,13 @@
         <v>1467</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0</v>
+        <v>3245.36</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1467</v>
+        <v>-1778.36</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>0</v>
+        <v>2.212242672119973</v>
       </c>
     </row>
     <row r="14">
@@ -3124,13 +3124,13 @@
         <v>51596.88</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>17685.83</v>
+        <v>30289.9</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>33911.05</v>
+        <v>21306.98</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.3427693690006062</v>
+        <v>0.587049061881261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-09-30 14:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -765,10 +765,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0</v>
+        <v>1846.35</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>0</v>
+        <v>325.23</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>0</v>
@@ -777,10 +777,10 @@
         <v>0</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>0</v>
+        <v>782.5599999999999</v>
       </c>
       <c r="M5" s="2" t="n">
-        <v>0</v>
+        <v>1284.32</v>
       </c>
       <c r="N5" s="2" t="n">
         <v>0</v>
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>4187.7</v>
+        <v>4283.4</v>
       </c>
       <c r="I12" s="2" t="n">
         <v>735.05</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>4016.57</v>
+        <v>8386.6</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -2026,14 +2026,14 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
+          <t>5 de 24</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
           <t>4 de 24</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>3 de 24</t>
-        </is>
-      </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
           <t>0 de 24</t>
@@ -2046,12 +2046,12 @@
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>1 de 24</t>
+          <t>2 de 24</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>3 de 24</t>
+          <t>4 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2188,7 +2188,7 @@
         <v>4847.61</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>4238.46</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>4000</v>
@@ -2431,7 +2431,7 @@
         <v>6827.71</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>8939.32</v>
+        <v>13405.05</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>5000</v>
@@ -2718,7 +2718,7 @@
         <v>43619.47</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>30289.9</v>
+        <v>38994.09</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>
@@ -2913,13 +2913,13 @@
         <v>5190</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>13436.79</v>
+        <v>15378.84</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>-8246.790000000001</v>
+        <v>-10188.84</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>2.588976878612717</v>
+        <v>2.963167630057804</v>
       </c>
     </row>
     <row r="8">
@@ -2937,13 +2937,13 @@
         <v>963</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>5420.96</v>
+        <v>5746.19</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>-4457.96</v>
+        <v>-4783.19</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5.629241952232606</v>
+        <v>5.966967808930425</v>
       </c>
     </row>
     <row r="9">
@@ -3057,13 +3057,13 @@
         <v>1467</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>3245.36</v>
+        <v>4027.92</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>-1778.36</v>
+        <v>-2560.92</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>2.212242672119973</v>
+        <v>2.745685071574642</v>
       </c>
     </row>
     <row r="14">
@@ -3081,13 +3081,13 @@
         <v>36556</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>8035.38</v>
+        <v>13689.73</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>28520.62</v>
+        <v>22866.27</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2198101542838385</v>
+        <v>0.3744865411970675</v>
       </c>
     </row>
     <row r="15">
@@ -3124,13 +3124,13 @@
         <v>51596.88</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>30289.9</v>
+        <v>38994.09</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>21306.98</v>
+        <v>12602.79</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.587049061881261</v>
+        <v>0.755745114820896</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-05 14:30:14
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1494,7 +1494,7 @@
         <v>0</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>1572.87</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>0 de 24</t>
+          <t>1 de 24</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2512,7 +2512,7 @@
         <v>9198.93</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0</v>
+        <v>1572.87</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6000</v>
@@ -2718,7 +2718,7 @@
         <v>71439.66</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>0</v>
+        <v>1572.87</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>45500</v>

</xml_diff>

<commit_message>
Actualización automática 2026-10-28 12:30:16
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>1006.25</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>3 de 24</t>
+          <t>4 de 24</t>
         </is>
       </c>
       <c r="N26" s="4" t="inlineStr">
@@ -2431,7 +2431,7 @@
         <v>13405.05</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>228.61</v>
+        <v>1234.86</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>6000</v>
@@ -2718,7 +2718,7 @@
         <v>71439.66</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>12662.01</v>
+        <v>13668.26</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>51500</v>
@@ -3081,13 +3081,13 @@
         <v>40549.17</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>11137.56</v>
+        <v>12143.81</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>29411.61</v>
+        <v>28405.36</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2746680141665045</v>
+        <v>0.2994835652616317</v>
       </c>
     </row>
     <row r="15">
@@ -3124,13 +3124,13 @@
         <v>51437.05</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>12662.01</v>
+        <v>13668.26</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>38775.04</v>
+        <v>37768.79</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2461651669370619</v>
+        <v>0.2657279140230631</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 11:30:19
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -1965,10 +1965,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>0</v>
+        <v>-160.88</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>0</v>
+        <v>-151.74</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0</v>
@@ -2701,7 +2701,7 @@
         <v>14166.93</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>270.91</v>
+        <v>-41.71</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>7000</v>
@@ -2718,7 +2718,7 @@
         <v>71439.66</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>13668.26</v>
+        <v>13355.64</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>51500</v>
@@ -2742,8 +2742,8 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2913,13 +2913,13 @@
         <v>700</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>-376.2</v>
+        <v>-537.08</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>1076.2</v>
+        <v>1237.08</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>-0.5374285714285714</v>
+        <v>-0.767257142857143</v>
       </c>
     </row>
     <row r="8">
@@ -2937,13 +2937,13 @@
         <v>300</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>228.61</v>
+        <v>76.87</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>71.38999999999999</v>
+        <v>223.13</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0.7620333333333333</v>
+        <v>0.2562333333333334</v>
       </c>
     </row>
     <row r="9">
@@ -3124,13 +3124,13 @@
         <v>51437.05</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13668.26</v>
+        <v>13355.64</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>37768.79</v>
+        <v>38081.41</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2657279140230631</v>
+        <v>0.2596501937805531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización automática 2026-10-29 17:30:17
</commit_message>
<xml_diff>
--- a/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
+++ b/data/HIDALGO HIDALGO PEDRO GUSTAVO.xlsx
@@ -894,7 +894,7 @@
         <v>0</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>17.91</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>327.77</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1006.25</v>
+        <v>4024.99</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
@@ -1494,13 +1494,13 @@
         <v>0</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>1572.87</v>
+        <v>1590.78</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="M17" s="2" t="n">
-        <v>8639.49</v>
+        <v>10651.98</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
@@ -2041,7 +2041,7 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>1 de 24</t>
+          <t>2 de 24</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2242,7 +2242,7 @@
         <v>9407.309999999999</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>327.77</v>
+        <v>345.68</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>6000</v>
@@ -2431,7 +2431,7 @@
         <v>13405.05</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1234.86</v>
+        <v>4253.6</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>6000</v>
@@ -2512,7 +2512,7 @@
         <v>9198.93</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>10212.36</v>
+        <v>12242.76</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>6000</v>
@@ -2718,7 +2718,7 @@
         <v>71439.66</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>13355.64</v>
+        <v>18422.69</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>51500</v>
@@ -3009,13 +3009,13 @@
         <v>407</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1572.87</v>
+        <v>1608.69</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>-1165.87</v>
+        <v>-1201.69</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3.864545454545454</v>
+        <v>3.952555282555283</v>
       </c>
     </row>
     <row r="12">
@@ -3081,13 +3081,13 @@
         <v>40549.17</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>12143.81</v>
+        <v>17175.04</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>28405.36</v>
+        <v>23374.13</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>0.2994835652616317</v>
+        <v>0.4235608275089232</v>
       </c>
     </row>
     <row r="15">
@@ -3124,13 +3124,13 @@
         <v>51437.05</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>13355.64</v>
+        <v>18422.69</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>38081.41</v>
+        <v>33014.36</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>0.2596501937805531</v>
+        <v>0.3581599255789358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>